<commit_message>
fix(slide11): resolve blank slide display and implement 3-Horizon Velocity Trilogy (Q3 vs H1 vs 2025)
</commit_message>
<xml_diff>
--- a/Egy_Nutri_Sales_Analysis_Template.xlsx
+++ b/Egy_Nutri_Sales_Analysis_Template.xlsx
@@ -19,14 +19,14 @@
     <sheet sheetId="13" name="Slide8_PediaStart1_Ranking" state="visible" r:id="rId16"/>
     <sheet sheetId="14" name="Slide9_PediaStart2_Ranking" state="visible" r:id="rId17"/>
     <sheet sheetId="15" name="Slide10_Quadrant_Matrix" state="visible" r:id="rId18"/>
-    <sheet sheetId="16" name="11-Q3 vs H1 Rep Velocity" state="visible" r:id="rId19"/>
+    <sheet sheetId="16" name="11-3-Horizon Rep Velocity" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="261">
   <si>
     <t>EGY NUTRI. - BUSINESS REVIEW &amp; SALES ANALYSIS MODEL</t>
   </si>
@@ -619,25 +619,34 @@
     <t>COMPANY STAR: Heavy volume, high growth exceeding company benchmark, expanding market share.</t>
   </si>
   <si>
-    <t>SLIDE 11: MEDICAL REP / ADM QUARTERLY VELOCITY (AVERAGE MONTHLY Q3 2026 vs H1 2026 BASELINE)</t>
-  </si>
-  <si>
-    <t>National Velocity Benchmark: H1 Monthly Avg = 138,315 cans/mo | Q3 Monthly Avg = 156,126 cans/mo | Acceleration = +12.9% (+17,811 cans/mo)</t>
+    <t>SLIDE 11: 3-HORIZON RUN-RATE VELOCITY: Q3 2026 vs H1 2026 BASELINE vs 2025 FULL YEAR</t>
+  </si>
+  <si>
+    <t>National Velocity Benchmark: 2025 MoAvg = 103,385 | H1 MoAvg = 138,315 | Q3 MoAvg = 156,126 | Acceleration vs H1 = +12.9% | Expansion vs '25 = +51.0%</t>
   </si>
   <si>
     <t>Medical Rep / ADM Name</t>
   </si>
   <si>
+    <t>2025 MoAvg</t>
+  </si>
+  <si>
     <t>H1 MoAvg (Jan-Jun)</t>
   </si>
   <si>
     <t>Q3 MoAvg (Jul-Sep)</t>
   </si>
   <si>
-    <t>Net Diff / Mo</t>
-  </si>
-  <si>
-    <t>Velocity %</t>
+    <t>Net Diff vs H1</t>
+  </si>
+  <si>
+    <t>Q3 vs H1 Vel.%</t>
+  </si>
+  <si>
+    <t>Q3 vs '25 Grw.%</t>
+  </si>
+  <si>
+    <t>Q3 Share %</t>
   </si>
   <si>
     <t>Performance Tier</t>
@@ -649,7 +658,7 @@
     <t>National Medical Rep Team Benchmark</t>
   </si>
   <si>
-    <t>Overall company run-rate accelerated by +12.9% in Q3</t>
+    <t>Overall company run-rate accelerated by +12.9% in Q3 (+51.0% vs 2025 baseline)</t>
   </si>
   <si>
     <t>Tier 1: High Accelerator 🚀</t>
@@ -676,7 +685,7 @@
     <t>Quarterly run-rate deceleration; urgent trade stock replenishment and rep detailing call review.</t>
   </si>
   <si>
-    <t>PRODUCT PORTFOLIO VELOCITY BREAKDOWN (Q3 2026 vs H1 2026)</t>
+    <t>PRODUCT PORTFOLIO 3-HORIZON VELOCITY BREAKDOWN (2025 vs H1 2026 vs Q3 2026)</t>
   </si>
   <si>
     <t>SKU Code</t>
@@ -688,13 +697,16 @@
     <t>Category</t>
   </si>
   <si>
-    <t>H1 MoAvg (Units)</t>
-  </si>
-  <si>
-    <t>Q3 MoAvg (Units)</t>
-  </si>
-  <si>
-    <t>Diff / Mo</t>
+    <t>2025 MoAvg (Baseline)</t>
+  </si>
+  <si>
+    <t>H1 MoAvg (Baseline)</t>
+  </si>
+  <si>
+    <t>Q3 MoAvg (Run-Rate)</t>
+  </si>
+  <si>
+    <t>Diff vs H1</t>
   </si>
   <si>
     <t>Supply / Demand Dynamic</t>
@@ -706,7 +718,7 @@
     <t>Core Infant</t>
   </si>
   <si>
-    <t>Strong demand (+10.5%), supply stable</t>
+    <t>Strong demand (+14.9% vs H1 | +60.7% vs '25), supply stable</t>
   </si>
   <si>
     <t>P2</t>
@@ -715,7 +727,7 @@
     <t>Core Follow-up</t>
   </si>
   <si>
-    <t>Slight dip (-8.4%) from peak Q2 promotions</t>
+    <t>Compounding steady run-rate (+5.9% vs H1 | +75.1% vs '25)</t>
   </si>
   <si>
     <t>PG3</t>
@@ -724,7 +736,7 @@
     <t>Growing Up Milk</t>
   </si>
   <si>
-    <t>Supply constraint in Q3 (-80.6%)</t>
+    <t>Temporary supply constraint in Q3 (-80.6% vs H1 | -70.5% vs '25)</t>
   </si>
   <si>
     <t>LF</t>
@@ -733,7 +745,7 @@
     <t>Specialty Lactose Free</t>
   </si>
   <si>
-    <t>Supply quota restricted (-46.2%)</t>
+    <t>Quota restricted in Q3 (-46.2% vs H1 | -24.1% vs '25)</t>
   </si>
   <si>
     <t>HA</t>
@@ -742,7 +754,7 @@
     <t>Specialty Hypoallergenic</t>
   </si>
   <si>
-    <t>Surge in hospital demand (+102.4%)</t>
+    <t>Surge in hospital demand (+102.4% vs H1 | +119.6% vs '25)</t>
   </si>
   <si>
     <t>AR</t>
@@ -751,7 +763,7 @@
     <t>Specialty Anti-Regurgitation</t>
   </si>
   <si>
-    <t>Steady pediatric adoption (+30.1%)</t>
+    <t>Steady pediatric adoption (+27.7% vs H1 | -3.8% vs '25)</t>
   </si>
   <si>
     <t>AC</t>
@@ -760,7 +772,7 @@
     <t>Specialty Anti-Colic</t>
   </si>
   <si>
-    <t>Massive surge across clinics (+101.9%)</t>
+    <t>Massive surge across clinics (+101.9% vs H1 | +188.5% vs '25)</t>
   </si>
   <si>
     <t>MUM</t>
@@ -769,7 +781,7 @@
     <t>Maternal Nutrition</t>
   </si>
   <si>
-    <t>Niche pharmacy detailing (-10.4%)</t>
+    <t>Niche pharmacy detailing (-19.3% vs H1 | -30.0% vs '25)</t>
   </si>
   <si>
     <t>PS1</t>
@@ -778,7 +790,7 @@
     <t>Economy Infant</t>
   </si>
   <si>
-    <t>Heavy clinic uptake across Upper Egypt (+35.7%)</t>
+    <t>Heavy clinic uptake in Upper Egypt (+35.7% vs H1 | +32.9% vs '25)</t>
   </si>
   <si>
     <t>PS2</t>
@@ -787,7 +799,7 @@
     <t>Economy Follow-up</t>
   </si>
   <si>
-    <t>Stable rural demand (-6.3%)</t>
+    <t>Stable rural demand (-4.9% vs H1 | +33.0% vs '25)</t>
   </si>
   <si>
     <t>LBW</t>
@@ -796,7 +808,7 @@
     <t>Specialty Low Birth Weight</t>
   </si>
   <si>
-    <t>Severe temporary stockout in Q3 (-98.8%)</t>
+    <t>Severe temporary stockout in Q3 (-99.2% vs H1)</t>
   </si>
 </sst>
 </file>
@@ -967,7 +979,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1038,13 +1050,14 @@
     </xf>
     <xf numFmtId="168" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="11" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -3628,18 +3641,18 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="44" customWidth="1"/>
+    <col min="4" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>197</v>
       </c>
@@ -3651,8 +3664,11 @@
       <c r="G1" s="23"/>
       <c r="H1" s="23"/>
       <c r="I1" s="23"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="47" t="s">
         <v>198</v>
       </c>
@@ -3664,8 +3680,11 @@
       <c r="G2" s="47"/>
       <c r="H2" s="47"/>
       <c r="I2" s="47"/>
-    </row>
-    <row r="3" ht="25" customHeight="1" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+    </row>
+    <row r="3" ht="25" customHeight="1" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>150</v>
       </c>
@@ -3693,8 +3712,17 @@
       <c r="I3" s="9" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J3" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" s="37" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
         <v>155</v>
       </c>
@@ -3702,28 +3730,37 @@
         <v>156</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D4" s="38">
+        <v>103385</v>
+      </c>
+      <c r="E4" s="38">
         <v>138315</v>
       </c>
-      <c r="E4" s="38">
+      <c r="F4" s="38">
         <v>156126</v>
       </c>
-      <c r="F4" s="48">
+      <c r="G4" s="48">
         <v>17811</v>
       </c>
-      <c r="G4" s="49">
+      <c r="H4" s="49">
         <v>0.12877128294111273</v>
       </c>
-      <c r="H4" s="37" t="s">
+      <c r="I4" s="49">
+        <v>0.5101417033418774</v>
+      </c>
+      <c r="J4" s="50">
+        <v>1</v>
+      </c>
+      <c r="K4" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="I4" s="37" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L4" s="37" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -3734,25 +3771,34 @@
         <v>75</v>
       </c>
       <c r="D5" s="12">
+        <v>7152</v>
+      </c>
+      <c r="E5" s="12">
         <v>8758</v>
       </c>
-      <c r="E5" s="12">
+      <c r="F5" s="12">
         <v>13898</v>
       </c>
-      <c r="F5" s="32">
+      <c r="G5" s="32">
         <v>5140</v>
       </c>
-      <c r="G5" s="50">
+      <c r="H5" s="51">
         <v>0.5868919844713405</v>
       </c>
-      <c r="H5" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="I5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="52">
+        <v>0.9432326621923937</v>
+      </c>
+      <c r="J5" s="13">
+        <v>0.08901784456144396</v>
+      </c>
+      <c r="K5" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="L5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -3763,25 +3809,34 @@
         <v>87</v>
       </c>
       <c r="D6" s="12">
+        <v>9337</v>
+      </c>
+      <c r="E6" s="12">
         <v>10461</v>
       </c>
-      <c r="E6" s="12">
+      <c r="F6" s="12">
         <v>15472</v>
       </c>
-      <c r="F6" s="32">
+      <c r="G6" s="32">
         <v>5011</v>
       </c>
-      <c r="G6" s="50">
+      <c r="H6" s="51">
         <v>0.47901730236115103</v>
       </c>
-      <c r="H6" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="I6" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="52">
+        <v>0.6570632965620649</v>
+      </c>
+      <c r="J6" s="13">
+        <v>0.0990994453198058</v>
+      </c>
+      <c r="K6" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="L6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -3792,25 +3847,34 @@
         <v>83</v>
       </c>
       <c r="D7" s="12">
+        <v>12877</v>
+      </c>
+      <c r="E7" s="12">
         <v>16459</v>
       </c>
-      <c r="E7" s="12">
+      <c r="F7" s="12">
         <v>23564</v>
       </c>
-      <c r="F7" s="32">
+      <c r="G7" s="32">
         <v>7105</v>
       </c>
-      <c r="G7" s="50">
+      <c r="H7" s="51">
         <v>0.43167871681147085</v>
       </c>
-      <c r="H7" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="I7" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="52">
+        <v>0.8299293313660014</v>
+      </c>
+      <c r="J7" s="13">
+        <v>0.15092937755402688</v>
+      </c>
+      <c r="K7" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="L7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -3821,25 +3885,34 @@
         <v>73</v>
       </c>
       <c r="D8" s="12">
+        <v>12441</v>
+      </c>
+      <c r="E8" s="12">
         <v>14302</v>
       </c>
-      <c r="E8" s="12">
+      <c r="F8" s="12">
         <v>18041</v>
       </c>
-      <c r="F8" s="32">
+      <c r="G8" s="32">
         <v>3739</v>
       </c>
-      <c r="G8" s="51">
+      <c r="H8" s="53">
         <v>0.26143196755698495</v>
       </c>
-      <c r="H8" s="52" t="s">
-        <v>210</v>
-      </c>
-      <c r="I8" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="52">
+        <v>0.4501245880556226</v>
+      </c>
+      <c r="J8" s="13">
+        <v>0.11555410373672546</v>
+      </c>
+      <c r="K8" s="54" t="s">
+        <v>213</v>
+      </c>
+      <c r="L8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -3850,25 +3923,34 @@
         <v>85</v>
       </c>
       <c r="D9" s="12">
+        <v>14859</v>
+      </c>
+      <c r="E9" s="12">
         <v>22305</v>
       </c>
-      <c r="E9" s="12">
+      <c r="F9" s="12">
         <v>25694</v>
       </c>
-      <c r="F9" s="32">
+      <c r="G9" s="32">
         <v>3389</v>
       </c>
-      <c r="G9" s="51">
+      <c r="H9" s="53">
         <v>0.15193902712396334</v>
       </c>
-      <c r="H9" s="52" t="s">
-        <v>210</v>
-      </c>
-      <c r="I9" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" s="52">
+        <v>0.7291876976916347</v>
+      </c>
+      <c r="J9" s="13">
+        <v>0.16457220450149238</v>
+      </c>
+      <c r="K9" s="54" t="s">
+        <v>213</v>
+      </c>
+      <c r="L9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -3879,25 +3961,34 @@
         <v>77</v>
       </c>
       <c r="D10" s="12">
+        <v>9951</v>
+      </c>
+      <c r="E10" s="12">
         <v>12895</v>
       </c>
-      <c r="E10" s="12">
+      <c r="F10" s="12">
         <v>13858</v>
       </c>
-      <c r="F10" s="32">
+      <c r="G10" s="32">
         <v>963</v>
       </c>
-      <c r="G10" s="53">
+      <c r="H10" s="55">
         <v>0.07468010856921281</v>
       </c>
-      <c r="H10" s="54" t="s">
-        <v>212</v>
-      </c>
-      <c r="I10" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" s="52">
+        <v>0.3926238568988041</v>
+      </c>
+      <c r="J10" s="13">
+        <v>0.08876164123848686</v>
+      </c>
+      <c r="K10" s="56" t="s">
+        <v>215</v>
+      </c>
+      <c r="L10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -3908,25 +3999,34 @@
         <v>71</v>
       </c>
       <c r="D11" s="12">
+        <v>7309</v>
+      </c>
+      <c r="E11" s="12">
         <v>10206</v>
       </c>
-      <c r="E11" s="12">
+      <c r="F11" s="12">
         <v>10314</v>
       </c>
-      <c r="F11" s="32">
+      <c r="G11" s="32">
         <v>108</v>
       </c>
-      <c r="G11" s="53">
+      <c r="H11" s="55">
         <v>0.010582010582010692</v>
       </c>
-      <c r="H11" s="54" t="s">
-        <v>212</v>
-      </c>
-      <c r="I11" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11" s="52">
+        <v>0.41113695443973186</v>
+      </c>
+      <c r="J11" s="13">
+        <v>0.06606202682448792</v>
+      </c>
+      <c r="K11" s="56" t="s">
+        <v>215</v>
+      </c>
+      <c r="L11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -3937,25 +4037,34 @@
         <v>79</v>
       </c>
       <c r="D12" s="12">
+        <v>15235</v>
+      </c>
+      <c r="E12" s="12">
         <v>20146</v>
       </c>
-      <c r="E12" s="12">
+      <c r="F12" s="12">
         <v>18614</v>
       </c>
-      <c r="F12" s="32">
+      <c r="G12" s="32">
         <v>-1532</v>
       </c>
-      <c r="G12" s="55">
+      <c r="H12" s="57">
         <v>-0.07604487243125191</v>
       </c>
-      <c r="H12" s="25" t="s">
-        <v>214</v>
-      </c>
-      <c r="I12" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I12" s="52">
+        <v>0.22179192648506718</v>
+      </c>
+      <c r="J12" s="13">
+        <v>0.1192242163380859</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>217</v>
+      </c>
+      <c r="L12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -3966,30 +4075,39 @@
         <v>81</v>
       </c>
       <c r="D13" s="12">
+        <v>14224</v>
+      </c>
+      <c r="E13" s="12">
         <v>22783</v>
       </c>
-      <c r="E13" s="12">
+      <c r="F13" s="12">
         <v>16671</v>
       </c>
-      <c r="F13" s="32">
+      <c r="G13" s="32">
         <v>-6112</v>
       </c>
-      <c r="G13" s="55">
+      <c r="H13" s="57">
         <v>-0.26827020146600533</v>
       </c>
-      <c r="H13" s="25" t="s">
-        <v>214</v>
-      </c>
-      <c r="I13" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I13" s="52">
+        <v>0.17203318335208095</v>
+      </c>
+      <c r="J13" s="13">
+        <v>0.10677913992544483</v>
+      </c>
+      <c r="K13" s="25" t="s">
+        <v>217</v>
+      </c>
+      <c r="L13" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
@@ -3998,360 +4116,471 @@
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
-    </row>
-    <row r="16" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+    </row>
+    <row r="16" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>203</v>
+        <v>226</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>223</v>
+        <v>204</v>
       </c>
       <c r="I16" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K16" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L16" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B17" t="s">
         <v>54</v>
       </c>
       <c r="C17" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D17" s="12">
+        <v>27891</v>
+      </c>
+      <c r="E17" s="12">
         <v>39024</v>
       </c>
-      <c r="E17" s="12">
+      <c r="F17" s="12">
         <v>44832</v>
       </c>
-      <c r="F17" s="32">
+      <c r="G17" s="32">
         <v>5808</v>
       </c>
-      <c r="G17" s="56">
+      <c r="H17" s="52">
         <v>0.14883148831488313</v>
       </c>
-      <c r="H17" t="s">
-        <v>226</v>
-      </c>
-      <c r="I17" t="s">
+      <c r="I17" s="52">
+        <v>0.6074002366354738</v>
+      </c>
+      <c r="J17" t="s">
+        <v>230</v>
+      </c>
+      <c r="K17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B18" t="s">
         <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D18" s="12">
+        <v>14775</v>
+      </c>
+      <c r="E18" s="12">
         <v>24418</v>
       </c>
-      <c r="E18" s="12">
+      <c r="F18" s="12">
         <v>25866</v>
       </c>
-      <c r="F18" s="32">
+      <c r="G18" s="32">
         <v>1448</v>
       </c>
-      <c r="G18" s="56">
+      <c r="H18" s="52">
         <v>0.05930051601277753</v>
       </c>
-      <c r="H18" t="s">
-        <v>229</v>
-      </c>
-      <c r="I18" t="s">
+      <c r="I18" s="52">
+        <v>0.7506598984771573</v>
+      </c>
+      <c r="J18" t="s">
+        <v>233</v>
+      </c>
+      <c r="K18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B19" t="s">
         <v>56</v>
       </c>
       <c r="C19" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D19" s="12">
+        <v>3515</v>
+      </c>
+      <c r="E19" s="12">
         <v>5338</v>
       </c>
-      <c r="E19" s="12">
+      <c r="F19" s="12">
         <v>1038</v>
       </c>
-      <c r="F19" s="32">
+      <c r="G19" s="32">
         <v>-4300</v>
       </c>
-      <c r="G19" s="57">
+      <c r="H19" s="58">
         <v>-0.8055451479955039</v>
       </c>
-      <c r="H19" t="s">
-        <v>232</v>
-      </c>
-      <c r="I19" t="s">
+      <c r="I19" s="52">
+        <v>-0.7046941678520626</v>
+      </c>
+      <c r="J19" t="s">
+        <v>236</v>
+      </c>
+      <c r="K19" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B20" t="s">
         <v>57</v>
       </c>
       <c r="C20" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D20" s="12">
+        <v>3073</v>
+      </c>
+      <c r="E20" s="12">
         <v>4335</v>
       </c>
-      <c r="E20" s="12">
+      <c r="F20" s="12">
         <v>2331</v>
       </c>
-      <c r="F20" s="32">
+      <c r="G20" s="32">
         <v>-2004</v>
       </c>
-      <c r="G20" s="57">
+      <c r="H20" s="58">
         <v>-0.46228373702422143</v>
       </c>
-      <c r="H20" t="s">
-        <v>235</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="I20" s="52">
+        <v>-0.24145785876993164</v>
+      </c>
+      <c r="J20" t="s">
+        <v>239</v>
+      </c>
+      <c r="K20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B21" t="s">
         <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D21" s="12">
+        <v>5436</v>
+      </c>
+      <c r="E21" s="12">
         <v>5899</v>
       </c>
-      <c r="E21" s="12">
+      <c r="F21" s="12">
         <v>11939</v>
       </c>
-      <c r="F21" s="32">
+      <c r="G21" s="32">
         <v>6040</v>
       </c>
-      <c r="G21" s="58">
+      <c r="H21" s="59">
         <v>1.0239023563315817</v>
       </c>
-      <c r="H21" t="s">
-        <v>238</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="I21" s="52">
+        <v>1.1962840323767474</v>
+      </c>
+      <c r="J21" t="s">
+        <v>242</v>
+      </c>
+      <c r="K21" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B22" t="s">
         <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D22" s="12">
+        <v>6203</v>
+      </c>
+      <c r="E22" s="12">
         <v>4676</v>
       </c>
-      <c r="E22" s="12">
+      <c r="F22" s="12">
         <v>5970</v>
       </c>
-      <c r="F22" s="32">
+      <c r="G22" s="32">
         <v>1294</v>
       </c>
-      <c r="G22" s="58">
+      <c r="H22" s="59">
         <v>0.27673224978614197</v>
       </c>
-      <c r="H22" t="s">
-        <v>241</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="I22" s="52">
+        <v>-0.03756246977269062</v>
+      </c>
+      <c r="J22" t="s">
+        <v>245</v>
+      </c>
+      <c r="K22" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B23" t="s">
         <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D23" s="12">
+        <v>5261</v>
+      </c>
+      <c r="E23" s="12">
         <v>7519</v>
       </c>
-      <c r="E23" s="12">
+      <c r="F23" s="12">
         <v>15180</v>
       </c>
-      <c r="F23" s="32">
+      <c r="G23" s="32">
         <v>7661</v>
       </c>
-      <c r="G23" s="58">
+      <c r="H23" s="59">
         <v>1.0188854900917677</v>
       </c>
-      <c r="H23" t="s">
-        <v>244</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="I23" s="52">
+        <v>1.8853830070328836</v>
+      </c>
+      <c r="J23" t="s">
+        <v>248</v>
+      </c>
+      <c r="K23" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B24" t="s">
         <v>61</v>
       </c>
       <c r="C24" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D24" s="12">
+        <v>833</v>
+      </c>
+      <c r="E24" s="12">
         <v>722</v>
       </c>
-      <c r="E24" s="12">
+      <c r="F24" s="12">
         <v>583</v>
       </c>
-      <c r="F24" s="32">
+      <c r="G24" s="32">
         <v>-139</v>
       </c>
-      <c r="G24" s="57">
+      <c r="H24" s="58">
         <v>-0.19252077562326875</v>
       </c>
-      <c r="H24" t="s">
-        <v>247</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="I24" s="52">
+        <v>-0.30012004801920766</v>
+      </c>
+      <c r="J24" t="s">
+        <v>251</v>
+      </c>
+      <c r="K24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B25" t="s">
         <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D25" s="12">
+        <v>24791</v>
+      </c>
+      <c r="E25" s="12">
         <v>24280</v>
       </c>
-      <c r="E25" s="12">
+      <c r="F25" s="12">
         <v>32950</v>
       </c>
-      <c r="F25" s="32">
+      <c r="G25" s="32">
         <v>8670</v>
       </c>
-      <c r="G25" s="58">
+      <c r="H25" s="59">
         <v>0.35708401976935744</v>
       </c>
-      <c r="H25" t="s">
-        <v>250</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="I25" s="52">
+        <v>0.329111371062079</v>
+      </c>
+      <c r="J25" t="s">
+        <v>254</v>
+      </c>
+      <c r="K25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B26" t="s">
         <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D26" s="12">
+        <v>11607</v>
+      </c>
+      <c r="E26" s="12">
         <v>16234</v>
       </c>
-      <c r="E26" s="12">
+      <c r="F26" s="12">
         <v>15438</v>
       </c>
-      <c r="F26" s="32">
+      <c r="G26" s="32">
         <v>-796</v>
       </c>
-      <c r="G26" s="57">
+      <c r="H26" s="58">
         <v>-0.04903289392632748</v>
       </c>
-      <c r="H26" t="s">
-        <v>253</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="I26" s="52">
+        <v>0.33005944688550004</v>
+      </c>
+      <c r="J26" t="s">
+        <v>257</v>
+      </c>
+      <c r="K26" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B27" t="s">
         <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D27" s="12">
+        <v>0</v>
+      </c>
+      <c r="E27" s="12">
         <v>5871</v>
       </c>
-      <c r="E27" s="12">
+      <c r="F27" s="12">
         <v>49</v>
       </c>
-      <c r="F27" s="32">
+      <c r="G27" s="32">
         <v>-5822</v>
       </c>
-      <c r="G27" s="57">
+      <c r="H27" s="58">
         <v>-0.9916538920115824</v>
       </c>
-      <c r="H27" t="s">
-        <v>256</v>
-      </c>
-      <c r="I27" t="s">
+      <c r="I27" s="52">
+        <v>1</v>
+      </c>
+      <c r="J27" t="s">
+        <v>260</v>
+      </c>
+      <c r="K27" t="s">
+        <v>15</v>
+      </c>
+      <c r="L27" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B15:L15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>